<commit_message>
fix(fichas): TMA alinea rangos de entrada (arribo 135-160, cierre 110-140) con los criterios del dictamen, evita conflicto celda-marca-X vs dictamen-CONFORME
</commit_message>
<xml_diff>
--- a/Proyectos Modelo/Proyecto_Carretera/TMA_TemperaturaAsfaltica.xlsx
+++ b/Proyectos Modelo/Proyecto_Carretera/TMA_TemperaturaAsfaltica.xlsx
@@ -473,7 +473,7 @@
         <v>Temperatura de arribo en obra</v>
       </c>
       <c r="E4" t="str">
-        <v>val-[2] // numerico-[140:155]:dec[1]:ej[145]</v>
+        <v>val-[2] // numerico-[135:160]:dec[1]:ej[145]</v>
       </c>
       <c r="F4" t="str">
         <v>Perfil de temperaturas in situ</v>
@@ -533,7 +533,7 @@
         <v>Temperatura de cierre de compactación</v>
       </c>
       <c r="E7" t="str">
-        <v>val-[5] // numerico-[110:120]:dec[1]:ej[115]</v>
+        <v>val-[5] // numerico-[110:140]:dec[1]:ej[115]</v>
       </c>
       <c r="F7" t="str">
         <v>Perfil de temperaturas in situ</v>

</xml_diff>